<commit_message>
Scrum: historias técnicas HT-01 a HT-08 y bitácora con los commits del sprint
- Product Backlog: hoja de historias técnicas (votación pendiente), sus 24 tarjetas y su lugar en el Sprint Backlog
- Tablero: las tareas transversales pasan a sus HT, cada una con su aceptación del PO (261 tareas)
- Bitácora: actividades con la hora de cada commit del repositorio
- equipo/henry.md: IDs actualizados (ClienteHttp = T-240, colección de Postman = T-245)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PtGmXDVgEBa1Hp6paBTjbG
</commit_message>
<xml_diff>
--- a/docs/scrum/SIGRO - Sprint 1 · Información del Sprint.xlsx
+++ b/docs/scrum/SIGRO - Sprint 1 · Información del Sprint.xlsx
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:F252"/>
+  <dimension ref="B2:F266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -566,7 +566,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>247 tareas · 29 HU · 153 puntos · del 15 al 28 de octubre de 2026 · todo en Done el lunes 27</t>
+          <t>261 tareas · 29 HU · 153 puntos · del 15 al 28 de octubre de 2026 · todo en Done el lunes 27</t>
         </is>
       </c>
     </row>
@@ -734,7 +734,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-004, T-006, T-234. 2 h · límite 26/10.</t>
+          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-004, T-006, T-240. 2 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -890,7 +890,7 @@
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-013, T-014, T-234. 2 h · límite 26/10.</t>
+          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-013, T-014, T-240. 2 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-030, T-031, T-234. 3 h · límite 26/10.</t>
+          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-030, T-031, T-240. 3 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 1 (app) y 20 (web) · Login: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-035, T-235. 3 h · límite 26/10.</t>
+          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 1 (app) y 20 (web) · Login: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-035, T-242. 3 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 10 · Usuarios, roles y dispositivos: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-057, T-235. 3 h · límite 26/10.</t>
+          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 10 · Usuarios, roles y dispositivos: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-057, T-242. 3 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -2416,7 +2416,7 @@
       </c>
       <c r="F98" s="7" t="inlineStr">
         <is>
-          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-091, T-092, T-234. 3 h · límite 26/10.</t>
+          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-091, T-092, T-240. 3 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="F106" s="7" t="inlineStr">
         <is>
-          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-099, T-100, T-234. 2 h · límite 26/10.</t>
+          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-099, T-100, T-240. 2 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="F122" s="7" t="inlineStr">
         <is>
-          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-114, T-116, T-234. 2 h · límite 26/10.</t>
+          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-114, T-116, T-240. 2 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -3040,7 +3040,7 @@
       </c>
       <c r="F130" s="7" t="inlineStr">
         <is>
-          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-123, T-124, T-234. 3 h · límite 26/10.</t>
+          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-123, T-124, T-240. 3 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -3200,7 +3200,7 @@
       </c>
       <c r="F138" s="7" t="inlineStr">
         <is>
-          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-131, T-132, T-234. 2 h · límite 26/10.</t>
+          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-131, T-132, T-240. 2 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -3356,7 +3356,7 @@
       </c>
       <c r="F146" s="7" t="inlineStr">
         <is>
-          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-139, T-140, T-234. 2 h · límite 26/10.</t>
+          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-139, T-140, T-240. 2 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -3512,7 +3512,7 @@
       </c>
       <c r="F154" s="7" t="inlineStr">
         <is>
-          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-147, T-148, T-234. 5 h · límite 26/10.</t>
+          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-147, T-148, T-240. 5 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="F162" s="7" t="inlineStr">
         <is>
-          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 14 · Recepción de compra: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-152, T-235. 4 h · límite 26/10.</t>
+          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 14 · Recepción de compra: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-152, T-242. 4 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="F163" s="7" t="inlineStr">
         <is>
-          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-155, T-156, T-234. 4 h · límite 26/10.</t>
+          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-155, T-156, T-240. 4 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -3809,7 +3809,7 @@
       </c>
       <c r="F169" s="7" t="inlineStr">
         <is>
-          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 3 · Salida y 4 · Ingreso (banda sin señal): botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-161, T-235. 14 h · límite 26/10.</t>
+          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 3 · Salida y 4 · Ingreso (banda sin señal): botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-161, T-242. 14 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -3965,7 +3965,7 @@
       </c>
       <c r="F177" s="7" t="inlineStr">
         <is>
-          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 8b · Envíos pendientes y 2 · Mis obras: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-167, T-235. 4 h · límite 26/10.</t>
+          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 8b · Envíos pendientes y 2 · Mis obras: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-167, T-242. 4 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -4121,7 +4121,7 @@
       </c>
       <c r="F185" s="7" t="inlineStr">
         <is>
-          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 3 · Registrar salida: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-175, T-235. 7 h · límite 26/10.</t>
+          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 3 · Registrar salida: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-175, T-242. 7 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -4296,7 +4296,7 @@
       </c>
       <c r="F194" s="7" t="inlineStr">
         <is>
-          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 5 · Consultar stock y 15 · Kárdex: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-183, T-235. 2 h · límite 26/10.</t>
+          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 5 · Consultar stock y 15 · Kárdex: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-183, T-242. 2 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="F195" s="7" t="inlineStr">
         <is>
-          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-186, T-188, T-234. 2 h · límite 26/10.</t>
+          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-186, T-188, T-240. 2 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="F203" s="7" t="inlineStr">
         <is>
-          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-196, T-197, T-234. 3 h · límite 26/10.</t>
+          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-196, T-197, T-240. 3 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -4787,7 +4787,7 @@
       </c>
       <c r="F219" s="7" t="inlineStr">
         <is>
-          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-212, T-213, T-234. 5 h · límite 26/10.</t>
+          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-212, T-213, T-240. 5 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="F227" s="7" t="inlineStr">
         <is>
-          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 6 · Registrar trabajador: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-217, T-235. 2 h · límite 26/10.</t>
+          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 6 · Registrar trabajador: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-217, T-242. 2 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -5103,7 +5103,7 @@
       </c>
       <c r="F235" s="7" t="inlineStr">
         <is>
-          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 7 · Asistencia de la jornada: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-225, T-235. 4 h · límite 26/10.</t>
+          <t>Nicolás programa la pantalla en android/ (Kotlin + Jetpack Compose) según la pantalla 7 · Asistencia de la jornada: botones grandes, una acción por pantalla, y lo que registra movimientos funciona sin señal. Empieza después de T-225, T-242. 4 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -5148,12 +5148,12 @@
     <row r="238" ht="66" customHeight="1">
       <c r="B238" s="4" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>HT. Historias técnicas (habilitadoras)</t>
         </is>
       </c>
       <c r="C238" s="5" t="inlineStr">
         <is>
-          <t>Tareas transversales (habilitan a todas las HU)</t>
+          <t>HT-01 · Desplegar el ambiente de pruebas (historia técnica · puntos por votar)</t>
         </is>
       </c>
       <c r="D238" s="6" t="inlineStr">
@@ -5174,26 +5174,30 @@
     </row>
     <row r="239" ht="66" customHeight="1">
       <c r="B239" s="8" t="n"/>
-      <c r="C239" s="8" t="n"/>
+      <c r="C239" s="9" t="n"/>
       <c r="D239" s="6" t="inlineStr">
         <is>
           <t>T-234</t>
         </is>
       </c>
-      <c r="E239" s="7" t="inlineStr">
-        <is>
-          <t>Programar el ClienteHttp para que la web hable con la API real (snake_case ↔ camelCase, errores {codigo, mensaje})</t>
+      <c r="E239" s="10" t="inlineStr">
+        <is>
+          <t>Aceptar HT-01 como Product Owner y moverla a Done</t>
         </is>
       </c>
       <c r="F239" s="7" t="inlineStr">
         <is>
-          <t>Henry: Habilitador de la web: una sola pieza que usan todas las pantallas para hablar con la API. Estado: To Do — desbloquea todas las tareas «Conectar…». 4 h · límite 26/10.</t>
+          <t>El Product Owner revisa HT-01 desde la interfaz, confirma la DoD (T1–T10) y la mueve a Done. Solo así cuenta en la velocidad del sprint. Estado: To Do — mueve la historia técnica a Done. 0.5 h · límite 27/10.</t>
         </is>
       </c>
     </row>
     <row r="240" ht="66" customHeight="1">
       <c r="B240" s="8" t="n"/>
-      <c r="C240" s="8" t="n"/>
+      <c r="C240" s="5" t="inlineStr">
+        <is>
+          <t>HT-02 · Configurar la integración continua (historia técnica · puntos por votar)</t>
+        </is>
+      </c>
       <c r="D240" s="6" t="inlineStr">
         <is>
           <t>T-235</t>
@@ -5201,37 +5205,41 @@
       </c>
       <c r="E240" s="7" t="inlineStr">
         <is>
-          <t>Crear el proyecto base de la app: Compose, Room, WorkManager y cliente de la API</t>
+          <t>Configurar las pruebas automáticas en cada PR con GitHub Actions</t>
         </is>
       </c>
       <c r="F240" s="7" t="inlineStr">
         <is>
-          <t>Nicolás: Habilitador de la app: el esqueleto sobre el que se construyen las pantallas del almacenero. Estado: To Do — desbloquea todas las tareas Android. 6 h · límite 26/10.</t>
+          <t>Adiel: Habilitador del equipo: sin esto ninguna HU puede cumplir la Definición de Terminado. Estado: To Do — T5 de la DoD. 3 h · límite 24/10.</t>
         </is>
       </c>
     </row>
     <row r="241" ht="66" customHeight="1">
       <c r="B241" s="8" t="n"/>
-      <c r="C241" s="8" t="n"/>
+      <c r="C241" s="9" t="n"/>
       <c r="D241" s="6" t="inlineStr">
         <is>
           <t>T-236</t>
         </is>
       </c>
-      <c r="E241" s="7" t="inlineStr">
-        <is>
-          <t>Cargar en la base las semillas de los 626 proveedores reales</t>
+      <c r="E241" s="10" t="inlineStr">
+        <is>
+          <t>Aceptar HT-02 como Product Owner y moverla a Done</t>
         </is>
       </c>
       <c r="F241" s="7" t="inlineStr">
         <is>
-          <t>Adiel implementa en api/ las clases de la HU —entidad, repositorio, servicio y controlador— con sus atributos y métodos; el servicio aplica la regla de negocio, el controlador verifica rol y obra en el servidor, y el endpoint queda documentado en api/LEEME.md con sus pruebas automáticas. 1 h · límite 25/10.</t>
+          <t>El Product Owner revisa HT-02 desde la interfaz, confirma la DoD (T1–T10) y la mueve a Done. Solo así cuenta en la velocidad del sprint. Estado: To Do — mueve la historia técnica a Done. 0.5 h · límite 27/10.</t>
         </is>
       </c>
     </row>
     <row r="242" ht="66" customHeight="1">
       <c r="B242" s="8" t="n"/>
-      <c r="C242" s="8" t="n"/>
+      <c r="C242" s="5" t="inlineStr">
+        <is>
+          <t>HT-03 · Proteger el repositorio y main (historia técnica · puntos por votar)</t>
+        </is>
+      </c>
       <c r="D242" s="6" t="inlineStr">
         <is>
           <t>T-237</t>
@@ -5239,12 +5247,12 @@
       </c>
       <c r="E242" s="7" t="inlineStr">
         <is>
-          <t>Configurar las pruebas automáticas en cada PR con GitHub Actions</t>
+          <t>Poner el repositorio en privado e invitar al docente como lector</t>
         </is>
       </c>
       <c r="F242" s="7" t="inlineStr">
         <is>
-          <t>Adiel: Habilitador del equipo: sin esto ninguna HU puede cumplir la Definición de Terminado. Estado: To Do — T5 de la DoD. 3 h · límite 24/10.</t>
+          <t>Fernando: Habilitador del equipo: sin esto ninguna HU puede cumplir la Definición de Terminado. Estado: To Do — hoy está público. 0.5 h · límite 24/10.</t>
         </is>
       </c>
     </row>
@@ -5258,37 +5266,41 @@
       </c>
       <c r="E243" s="7" t="inlineStr">
         <is>
-          <t>Poner el repositorio en privado e invitar al docente como lector</t>
+          <t>Proteger la rama main: PR obligatorio con una aprobación de otro integrante</t>
         </is>
       </c>
       <c r="F243" s="7" t="inlineStr">
         <is>
-          <t>Fernando: Trabajo del Scrum Master para que el equipo y el docente vean el avance real. Estado: To Do — hoy está público. 0.5 h · límite 23/10.</t>
+          <t>Fernando: Habilitador del equipo: sin esto ninguna HU puede cumplir la Definición de Terminado. 0.5 h · límite 24/10.</t>
         </is>
       </c>
     </row>
     <row r="244" ht="66" customHeight="1">
       <c r="B244" s="8" t="n"/>
-      <c r="C244" s="8" t="n"/>
+      <c r="C244" s="9" t="n"/>
       <c r="D244" s="6" t="inlineStr">
         <is>
           <t>T-239</t>
         </is>
       </c>
-      <c r="E244" s="7" t="inlineStr">
-        <is>
-          <t>Armar el tablero en GitHub Projects con las plantillas de DoR y DoD</t>
+      <c r="E244" s="10" t="inlineStr">
+        <is>
+          <t>Aceptar HT-03 como Product Owner y moverla a Done</t>
         </is>
       </c>
       <c r="F244" s="7" t="inlineStr">
         <is>
-          <t>Fernando: Trabajo del Scrum Master para que el equipo y el docente vean el avance real. Estado: Doing. 2 h · límite 23/10.</t>
+          <t>El Product Owner revisa HT-03 desde la interfaz, confirma la DoD (T1–T10) y la mueve a Done. Solo así cuenta en la velocidad del sprint. Estado: To Do — mueve la historia técnica a Done. 0.5 h · límite 27/10.</t>
         </is>
       </c>
     </row>
     <row r="245" ht="66" customHeight="1">
       <c r="B245" s="8" t="n"/>
-      <c r="C245" s="8" t="n"/>
+      <c r="C245" s="5" t="inlineStr">
+        <is>
+          <t>HT-04 · Conectar la web con la API real (historia técnica · puntos por votar)</t>
+        </is>
+      </c>
       <c r="D245" s="6" t="inlineStr">
         <is>
           <t>T-240</t>
@@ -5296,37 +5308,41 @@
       </c>
       <c r="E245" s="7" t="inlineStr">
         <is>
-          <t>Facilitar el Daily Scrum de 15 minutos cada día, registrarlo y actualizar el burndown</t>
+          <t>Programar el ClienteHttp para que la web hable con la API real (snake_case ↔ camelCase, errores {codigo, mensaje})</t>
         </is>
       </c>
       <c r="F245" s="7" t="inlineStr">
         <is>
-          <t>Fernando: Trabajo del Scrum Master para que el equipo y el docente vean el avance real. Estado: Doing — hasta el 28/10. 2 h · límite 27/10.</t>
+          <t>Henry: Habilitador de la web: una sola pieza que usan todas las pantallas para hablar con la API. Estado: To Do — desbloquea todas las tareas «Conectar…». 4 h · límite 26/10.</t>
         </is>
       </c>
     </row>
     <row r="246" ht="66" customHeight="1">
       <c r="B246" s="8" t="n"/>
-      <c r="C246" s="8" t="n"/>
+      <c r="C246" s="9" t="n"/>
       <c r="D246" s="6" t="inlineStr">
         <is>
           <t>T-241</t>
         </is>
       </c>
-      <c r="E246" s="7" t="inlineStr">
-        <is>
-          <t>Simplificar los textos de cada pantalla web: título y una línea, con ayuda «?» bajo demanda</t>
+      <c r="E246" s="10" t="inlineStr">
+        <is>
+          <t>Aceptar HT-04 como Product Owner y moverla a Done</t>
         </is>
       </c>
       <c r="F246" s="7" t="inlineStr">
         <is>
-          <t>Fernando: Para que la gente de SEVENS entienda y use el sistema sin una capacitación larga. Estado: To Do — observación de Fernando: hoy hay demasiado texto. 3 h · límite 26/10.</t>
+          <t>El Product Owner revisa HT-04 desde la interfaz, confirma la DoD (T1–T10) y la mueve a Done. Solo así cuenta en la velocidad del sprint. Estado: To Do — mueve la historia técnica a Done. 0.5 h · límite 27/10.</t>
         </is>
       </c>
     </row>
     <row r="247" ht="66" customHeight="1">
       <c r="B247" s="8" t="n"/>
-      <c r="C247" s="8" t="n"/>
+      <c r="C247" s="5" t="inlineStr">
+        <is>
+          <t>HT-05 · Crear la base de la app Android (historia técnica · puntos por votar)</t>
+        </is>
+      </c>
       <c r="D247" s="6" t="inlineStr">
         <is>
           <t>T-242</t>
@@ -5334,37 +5350,41 @@
       </c>
       <c r="E247" s="7" t="inlineStr">
         <is>
-          <t>Validar las pantallas con el cliente (Pool) en una sesión corta y registrar sus observaciones</t>
+          <t>Crear el proyecto base de la app: Compose, Room, WorkManager y cliente de la API</t>
         </is>
       </c>
       <c r="F247" s="7" t="inlineStr">
         <is>
-          <t>Fernando: Para que la gente de SEVENS entienda y use el sistema sin una capacitación larga. Estado: To Do — que lo use quien lo va a usar. 1.5 h · límite 26/10.</t>
+          <t>Nicolás: Habilitador de la app: el esqueleto sobre el que se construyen las pantallas del almacenero. Estado: To Do — desbloquea todas las tareas Android. 6 h · límite 26/10.</t>
         </is>
       </c>
     </row>
     <row r="248" ht="66" customHeight="1">
       <c r="B248" s="8" t="n"/>
-      <c r="C248" s="8" t="n"/>
+      <c r="C248" s="9" t="n"/>
       <c r="D248" s="6" t="inlineStr">
         <is>
           <t>T-243</t>
         </is>
       </c>
-      <c r="E248" s="7" t="inlineStr">
-        <is>
-          <t>Revisar la app con guantes y al sol: botones grandes, una acción por pantalla, contraste AA</t>
+      <c r="E248" s="10" t="inlineStr">
+        <is>
+          <t>Aceptar HT-05 como Product Owner y moverla a Done</t>
         </is>
       </c>
       <c r="F248" s="7" t="inlineStr">
         <is>
-          <t>Nicolás: Para que la gente de SEVENS entienda y use el sistema sin una capacitación larga. Estado: To Do — el almacenero trabaja en obra. 2 h · límite 26/10.</t>
+          <t>El Product Owner revisa HT-05 desde la interfaz, confirma la DoD (T1–T10) y la mueve a Done. Solo así cuenta en la velocidad del sprint. Estado: To Do — mueve la historia técnica a Done. 0.5 h · límite 27/10.</t>
         </is>
       </c>
     </row>
     <row r="249" ht="66" customHeight="1">
       <c r="B249" s="8" t="n"/>
-      <c r="C249" s="8" t="n"/>
+      <c r="C249" s="5" t="inlineStr">
+        <is>
+          <t>HT-06 · Publicar el contrato de la API y Postman (historia técnica · puntos por votar)</t>
+        </is>
+      </c>
       <c r="D249" s="6" t="inlineStr">
         <is>
           <t>T-244</t>
@@ -5372,12 +5392,12 @@
       </c>
       <c r="E249" s="7" t="inlineStr">
         <is>
-          <t>Modelar los 3 diagramas de casos de uso y los 3 de secuencia (importación S10, salida sin señal, recepción y costo promedio)</t>
+          <t>Publicar el OpenAPI de la API en el ambiente de pruebas</t>
         </is>
       </c>
       <c r="F249" s="7" t="inlineStr">
         <is>
-          <t>Fernando dibuja el diagrama UML que explica cómo funciona la HU (actores, pantallas, API y base) para que quien programa no tenga que adivinar el flujo. Estado: Done — en el lienzo; cubren HU-07, 35, 37, 38, 40 y 55. 2 h · límite 24/10.</t>
+          <t>Adiel implementa en api/ las clases de la HU —entidad, repositorio, servicio y controlador— con sus atributos y métodos; el servicio aplica la regla de negocio, el controlador verifica rol y obra en el servidor, y el endpoint queda documentado en api/LEEME.md con sus pruebas automáticas. Estado: Doing — Swagger de FastAPI ya existe en local. 1 h · límite 25/10.</t>
         </is>
       </c>
     </row>
@@ -5391,55 +5411,337 @@
       </c>
       <c r="E250" s="7" t="inlineStr">
         <is>
-          <t>Dibujar los diagramas de actividades del negocio y de estados</t>
+          <t>Armar y compartir la colección de Postman con entorno de pruebas, login y un ejemplo correcto y uno de error por endpoint</t>
         </is>
       </c>
       <c r="F250" s="7" t="inlineStr">
         <is>
-          <t>Nicolás dibuja el diagrama UML que explica cómo funciona la HU (actores, pantallas, API y base) para que quien programa no tenga que adivinar el flujo. Estado: Done — 14 hojas: A1–A4 y E1–E3 (22/10). 2 h · límite 24/10.</t>
+          <t>Henry, que no programó lo que falta de HT-06, prueba los endpoints con Postman y la interfaz contra cada condición final de la tarjeta 3 en el ambiente de pruebas; si todo cumple aprueba el PR, si no lo devuelve con la falla. 3 h · límite 24/10.</t>
         </is>
       </c>
     </row>
     <row r="251" ht="66" customHeight="1">
       <c r="B251" s="8" t="n"/>
-      <c r="C251" s="8" t="n"/>
+      <c r="C251" s="9" t="n"/>
       <c r="D251" s="6" t="inlineStr">
         <is>
           <t>T-246</t>
         </is>
       </c>
-      <c r="E251" s="7" t="inlineStr">
+      <c r="E251" s="10" t="inlineStr">
+        <is>
+          <t>Aceptar HT-06 como Product Owner y moverla a Done</t>
+        </is>
+      </c>
+      <c r="F251" s="7" t="inlineStr">
+        <is>
+          <t>El Product Owner revisa HT-06 desde la interfaz, confirma la DoD (T1–T10) y la mueve a Done. Solo así cuenta en la velocidad del sprint. Estado: To Do — mueve la historia técnica a Done. 0.5 h · límite 27/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="252" ht="66" customHeight="1">
+      <c r="B252" s="8" t="n"/>
+      <c r="C252" s="5" t="inlineStr">
+        <is>
+          <t>HT-07 · Cargar los datos de prueba reales (historia técnica · puntos por votar)</t>
+        </is>
+      </c>
+      <c r="D252" s="6" t="inlineStr">
+        <is>
+          <t>T-247</t>
+        </is>
+      </c>
+      <c r="E252" s="7" t="inlineStr">
+        <is>
+          <t>Cargar en la base los 626 proveedores y el catálogo de insumos del cliente</t>
+        </is>
+      </c>
+      <c r="F252" s="7" t="inlineStr">
+        <is>
+          <t>Adiel implementa en api/ las clases de la HU —entidad, repositorio, servicio y controlador— con sus atributos y métodos; el servicio aplica la regla de negocio, el controlador verifica rol y obra en el servidor, y el endpoint queda documentado en api/LEEME.md con sus pruebas automáticas. Estado: To Do — cargador idempotente ya probado. 1 h · límite 25/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="253" ht="66" customHeight="1">
+      <c r="B253" s="8" t="n"/>
+      <c r="C253" s="8" t="n"/>
+      <c r="D253" s="6" t="inlineStr">
+        <is>
+          <t>T-248</t>
+        </is>
+      </c>
+      <c r="E253" s="7" t="inlineStr">
+        <is>
+          <t>Crear la obra Multifamiliar Flores con su relación de insumos del S10 en la base de pruebas</t>
+        </is>
+      </c>
+      <c r="F253" s="7" t="inlineStr">
+        <is>
+          <t>Adiel implementa en api/ las clases de la HU —entidad, repositorio, servicio y controlador— con sus atributos y métodos; el servicio aplica la regla de negocio, el controlador verifica rol y obra en el servidor, y el endpoint queda documentado en api/LEEME.md con sus pruebas automáticas. 1 h · límite 25/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="254" ht="66" customHeight="1">
+      <c r="B254" s="8" t="n"/>
+      <c r="C254" s="9" t="n"/>
+      <c r="D254" s="6" t="inlineStr">
+        <is>
+          <t>T-249</t>
+        </is>
+      </c>
+      <c r="E254" s="10" t="inlineStr">
+        <is>
+          <t>Aceptar HT-07 como Product Owner y moverla a Done</t>
+        </is>
+      </c>
+      <c r="F254" s="7" t="inlineStr">
+        <is>
+          <t>El Product Owner revisa HT-07 desde la interfaz, confirma la DoD (T1–T10) y la mueve a Done. Solo así cuenta en la velocidad del sprint. Estado: To Do — mueve la historia técnica a Done. 0.5 h · límite 27/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="255" ht="66" customHeight="1">
+      <c r="B255" s="8" t="n"/>
+      <c r="C255" s="5" t="inlineStr">
+        <is>
+          <t>HT-08 · Autenticar a los servicios entre sí (historia técnica · puntos por votar)</t>
+        </is>
+      </c>
+      <c r="D255" s="6" t="inlineStr">
+        <is>
+          <t>T-250</t>
+        </is>
+      </c>
+      <c r="E255" s="7" t="inlineStr">
+        <is>
+          <t>Exigir el token de servicio en Integraciones</t>
+        </is>
+      </c>
+      <c r="F255" s="7" t="inlineStr">
+        <is>
+          <t>Fernando conecta con el sistema externo sin que la API dependa de él: el microservicio devuelve datos normalizados y, si el servicio cae, el registro no se bloquea. Se prueba con el archivo o servicio real. Estado: Done — X-Servicio-Token, 22/10. 1 h · límite 25/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="256" ht="66" customHeight="1">
+      <c r="B256" s="8" t="n"/>
+      <c r="C256" s="8" t="n"/>
+      <c r="D256" s="6" t="inlineStr">
+        <is>
+          <t>T-251</t>
+        </is>
+      </c>
+      <c r="E256" s="7" t="inlineStr">
+        <is>
+          <t>Configurar el token de servicio en docker compose y enviarlo desde la API a Integraciones y Notificaciones</t>
+        </is>
+      </c>
+      <c r="F256" s="7" t="inlineStr">
+        <is>
+          <t>Adiel: Habilitador del equipo: sin esto ninguna HU puede cumplir la Definición de Terminado. 1.5 h · límite 24/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="257" ht="66" customHeight="1">
+      <c r="B257" s="9" t="n"/>
+      <c r="C257" s="9" t="n"/>
+      <c r="D257" s="6" t="inlineStr">
+        <is>
+          <t>T-252</t>
+        </is>
+      </c>
+      <c r="E257" s="10" t="inlineStr">
+        <is>
+          <t>Aceptar HT-08 como Product Owner y moverla a Done</t>
+        </is>
+      </c>
+      <c r="F257" s="7" t="inlineStr">
+        <is>
+          <t>El Product Owner revisa HT-08 desde la interfaz, confirma la DoD (T1–T10) y la mueve a Done. Solo así cuenta en la velocidad del sprint. Estado: To Do — mueve la historia técnica a Done. 0.5 h · límite 27/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="258" ht="66" customHeight="1">
+      <c r="B258" s="4" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C258" s="5" t="inlineStr">
+        <is>
+          <t>Otras tareas transversales</t>
+        </is>
+      </c>
+      <c r="D258" s="6" t="inlineStr">
+        <is>
+          <t>T-253</t>
+        </is>
+      </c>
+      <c r="E258" s="7" t="inlineStr">
+        <is>
+          <t>Armar el tablero en GitHub Projects con las plantillas de DoR y DoD</t>
+        </is>
+      </c>
+      <c r="F258" s="7" t="inlineStr">
+        <is>
+          <t>Fernando: Trabajo del Scrum Master para que el equipo y el docente vean el avance real. Estado: Doing. 2 h · límite 23/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="259" ht="66" customHeight="1">
+      <c r="B259" s="8" t="n"/>
+      <c r="C259" s="8" t="n"/>
+      <c r="D259" s="6" t="inlineStr">
+        <is>
+          <t>T-254</t>
+        </is>
+      </c>
+      <c r="E259" s="7" t="inlineStr">
+        <is>
+          <t>Facilitar el Daily Scrum de 15 minutos cada día, registrarlo y actualizar el burndown</t>
+        </is>
+      </c>
+      <c r="F259" s="7" t="inlineStr">
+        <is>
+          <t>Fernando: Trabajo del Scrum Master para que el equipo y el docente vean el avance real. Estado: Doing — hasta el 28/10. 2 h · límite 27/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="260" ht="66" customHeight="1">
+      <c r="B260" s="8" t="n"/>
+      <c r="C260" s="8" t="n"/>
+      <c r="D260" s="6" t="inlineStr">
+        <is>
+          <t>T-255</t>
+        </is>
+      </c>
+      <c r="E260" s="7" t="inlineStr">
+        <is>
+          <t>Simplificar los textos de cada pantalla web: título y una línea, con ayuda «?» bajo demanda</t>
+        </is>
+      </c>
+      <c r="F260" s="7" t="inlineStr">
+        <is>
+          <t>Fernando: Para que la gente de SEVENS entienda y use el sistema sin una capacitación larga. Estado: To Do — observación de Fernando: hoy hay demasiado texto. 3 h · límite 26/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="261" ht="66" customHeight="1">
+      <c r="B261" s="8" t="n"/>
+      <c r="C261" s="8" t="n"/>
+      <c r="D261" s="6" t="inlineStr">
+        <is>
+          <t>T-256</t>
+        </is>
+      </c>
+      <c r="E261" s="7" t="inlineStr">
+        <is>
+          <t>Validar las pantallas con el cliente (Pool) en una sesión corta y registrar sus observaciones</t>
+        </is>
+      </c>
+      <c r="F261" s="7" t="inlineStr">
+        <is>
+          <t>Fernando: Para que la gente de SEVENS entienda y use el sistema sin una capacitación larga. Estado: To Do — que lo use quien lo va a usar. 1.5 h · límite 26/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="262" ht="66" customHeight="1">
+      <c r="B262" s="8" t="n"/>
+      <c r="C262" s="8" t="n"/>
+      <c r="D262" s="6" t="inlineStr">
+        <is>
+          <t>T-257</t>
+        </is>
+      </c>
+      <c r="E262" s="7" t="inlineStr">
+        <is>
+          <t>Revisar la app con guantes y al sol: botones grandes, una acción por pantalla, contraste AA</t>
+        </is>
+      </c>
+      <c r="F262" s="7" t="inlineStr">
+        <is>
+          <t>Nicolás: Para que la gente de SEVENS entienda y use el sistema sin una capacitación larga. Estado: To Do — el almacenero trabaja en obra. 2 h · límite 26/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="263" ht="66" customHeight="1">
+      <c r="B263" s="8" t="n"/>
+      <c r="C263" s="8" t="n"/>
+      <c r="D263" s="6" t="inlineStr">
+        <is>
+          <t>T-258</t>
+        </is>
+      </c>
+      <c r="E263" s="7" t="inlineStr">
+        <is>
+          <t>Modelar los 3 diagramas de casos de uso y los 3 de secuencia (importación S10, salida sin señal, recepción y costo promedio)</t>
+        </is>
+      </c>
+      <c r="F263" s="7" t="inlineStr">
+        <is>
+          <t>Fernando dibuja el diagrama UML que explica cómo funciona la HU (actores, pantallas, API y base) para que quien programa no tenga que adivinar el flujo. Estado: Done — en el lienzo; cubren HU-07, 35, 37, 38, 40 y 55. 2 h · límite 24/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="264" ht="66" customHeight="1">
+      <c r="B264" s="8" t="n"/>
+      <c r="C264" s="8" t="n"/>
+      <c r="D264" s="6" t="inlineStr">
+        <is>
+          <t>T-259</t>
+        </is>
+      </c>
+      <c r="E264" s="7" t="inlineStr">
+        <is>
+          <t>Dibujar los diagramas de actividades del negocio y de estados</t>
+        </is>
+      </c>
+      <c r="F264" s="7" t="inlineStr">
+        <is>
+          <t>Nicolás dibuja el diagrama UML que explica cómo funciona la HU (actores, pantallas, API y base) para que quien programa no tenga que adivinar el flujo. Estado: Done — 14 hojas: A1–A4 y E1–E3 (22/10). 2 h · límite 24/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="265" ht="66" customHeight="1">
+      <c r="B265" s="8" t="n"/>
+      <c r="C265" s="8" t="n"/>
+      <c r="D265" s="6" t="inlineStr">
+        <is>
+          <t>T-260</t>
+        </is>
+      </c>
+      <c r="E265" s="7" t="inlineStr">
         <is>
           <t>Dibujar la arquitectura en las cuatro vistas del C4 a partir del diagrama de microservicios</t>
         </is>
       </c>
-      <c r="F251" s="7" t="inlineStr">
+      <c r="F265" s="7" t="inlineStr">
         <is>
           <t>Nicolás dibuja el diagrama UML que explica cómo funciona la HU (actores, pantallas, API y base) para que quien programa no tenga que adivinar el flujo. Estado: To Do — parte de api/docs/diagrama-microservicios.png. 4 h · límite 24/10.</t>
         </is>
       </c>
     </row>
-    <row r="252" ht="66" customHeight="1">
-      <c r="B252" s="9" t="n"/>
-      <c r="C252" s="9" t="n"/>
-      <c r="D252" s="6" t="inlineStr">
-        <is>
-          <t>T-247</t>
-        </is>
-      </c>
-      <c r="E252" s="7" t="inlineStr">
+    <row r="266" ht="66" customHeight="1">
+      <c r="B266" s="9" t="n"/>
+      <c r="C266" s="9" t="n"/>
+      <c r="D266" s="6" t="inlineStr">
+        <is>
+          <t>T-261</t>
+        </is>
+      </c>
+      <c r="E266" s="7" t="inlineStr">
         <is>
           <t>Preparar la demo de la Sprint Review: una compra que cruza recepción, salida y costo de punta a punta</t>
         </is>
       </c>
-      <c r="F252" s="7" t="inlineStr">
+      <c r="F266" s="7" t="inlineStr">
         <is>
           <t>Fernando: Demostración para el cliente y el docente en la Sprint Review del 28/10. 2 h · límite 27/10.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="37">
+  <mergeCells count="46">
     <mergeCell ref="C109:C115"/>
     <mergeCell ref="B166:B205"/>
     <mergeCell ref="C149:C156"/>
@@ -5447,9 +5749,10 @@
     <mergeCell ref="C101:C108"/>
     <mergeCell ref="C166:C171"/>
     <mergeCell ref="C55:C61"/>
+    <mergeCell ref="B258:B266"/>
     <mergeCell ref="C15:C22"/>
+    <mergeCell ref="C249:C251"/>
     <mergeCell ref="C62:C69"/>
-    <mergeCell ref="B238:B252"/>
     <mergeCell ref="C141:C148"/>
     <mergeCell ref="C172:C179"/>
     <mergeCell ref="C23:C31"/>
@@ -5462,21 +5765,29 @@
     <mergeCell ref="B222:B237"/>
     <mergeCell ref="C85:C92"/>
     <mergeCell ref="C230:C237"/>
+    <mergeCell ref="C238:C239"/>
     <mergeCell ref="C93:C100"/>
-    <mergeCell ref="C238:C252"/>
+    <mergeCell ref="C247:C248"/>
+    <mergeCell ref="B133:B165"/>
     <mergeCell ref="C40:C47"/>
     <mergeCell ref="B70:B132"/>
-    <mergeCell ref="B133:B165"/>
     <mergeCell ref="C214:C221"/>
+    <mergeCell ref="C258:C266"/>
+    <mergeCell ref="C240:C241"/>
     <mergeCell ref="C157:C165"/>
     <mergeCell ref="C133:C140"/>
     <mergeCell ref="C222:C229"/>
     <mergeCell ref="C6:C14"/>
     <mergeCell ref="C198:C205"/>
+    <mergeCell ref="C252:C254"/>
     <mergeCell ref="C70:C77"/>
+    <mergeCell ref="C255:C257"/>
+    <mergeCell ref="C242:C244"/>
     <mergeCell ref="C188:C197"/>
+    <mergeCell ref="C245:C246"/>
     <mergeCell ref="C116:C124"/>
     <mergeCell ref="C32:C39"/>
+    <mergeCell ref="B238:B257"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -5866,7 +6177,7 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Pasarlo a privado e invitar al docente como lector (T-238)</t>
+          <t>Pasarlo a privado e invitar al docente como lector (T-237)</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
@@ -6228,7 +6539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:H22"/>
+  <dimension ref="B1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -6445,7 +6756,7 @@
       <c r="F12" s="7" t="inlineStr"/>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Planning Poker: estimación de las historias con votación de los cuatro integrantes</t>
+          <t>Planning Poker: estimación de las historias con el voto de los cuatro integrantes</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -6516,52 +6827,56 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>T-245</t>
+          <t>T-259</t>
         </is>
       </c>
     </row>
     <row r="15" ht="40" customHeight="1">
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Día 8</t>
+          <t>Día 7</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Víctor Adiel Luján</t>
+          <t>Fernando Istaña</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Product Owner / backend</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr"/>
+          <t>Scrum Master</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>19:02</t>
+        </is>
+      </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>API con login, roles, obras, asignaciones, dispositivos, proveedores, compras y tareo (629 pruebas), microservicio de Notificaciones y diagramas físico y entidad-relación</t>
+          <t>Subir al repositorio el contexto del proyecto, las historias del Sprint 1 y 2 y las reglas de dominio (commit)</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>HU-01, 12–15, 29, 30, 32, 62, 63</t>
+          <t>CLAUDE.md, docs/</t>
         </is>
       </c>
     </row>
     <row r="16" ht="40" customHeight="1">
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Día 8</t>
+          <t>Día 7</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -6571,18 +6886,22 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Developer (integraciones)</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr"/>
+          <t>Scrum Master</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>20:33</t>
+        </is>
+      </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Importador del S10: lector de la Relación de insumos (284 insumos, 0 fallidos) y consulta de DNI</t>
+          <t>Subir las pantallas del Sprint 1, la estimación del equipo y los entregables (commit)</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>T-023</t>
+          <t>Diseño UI</t>
         </is>
       </c>
     </row>
@@ -6604,18 +6923,22 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Developer (web)</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr"/>
+          <t>Developer (web e integraciones)</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Pantallas web: catálogo (2 243 insumos), proveedores (626), compras y recepción, reposición, kárdex y reverso, obra activa y accesibilidad</t>
+          <t>Web de oficina (pantallas e importador del S10), microservicio de integraciones (RUC, DNI, S10: 284 insumos, 0 fallidos), semillas reales del cliente y documentos Scrum (commit)</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>HU-08, 23, 24, 26, 27, 29, 30, 32, 35, 43, 45, 57</t>
+          <t>T-023</t>
         </is>
       </c>
     </row>
@@ -6632,23 +6955,27 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Fernando Istaña</t>
+          <t>Víctor Adiel Luján</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Scrum Master</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr"/>
+          <t>Product Owner / backend</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Diseño de las 23 pantallas del Sprint 1, casos de uso y diagramas de secuencia</t>
+          <t>API de obra, compras y tareo (629 pruebas) y microservicio de Notificaciones con outbox; PR #1 fusionado</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>Diseño UI y Modelado UML</t>
+          <t>HU-01, 12–15, 29, 30, 32, 62, 63</t>
         </is>
       </c>
     </row>
@@ -6665,23 +6992,27 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Equipo Scrum</t>
+          <t>Víctor Adiel Luján</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Scrum Team</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr"/>
+          <t>Product Owner / backend</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Presentación al docente: puntuación de las HU, objetivo del sprint y tarjetas DoR y DoD; se recibe su retroalimentación</t>
+          <t>Diagramas físico (con outbox), entidad-relación y esquema de microservicios (commit)</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>Product Backlog y Sprint Backlog</t>
+          <t>Base de datos</t>
         </is>
       </c>
     </row>
@@ -6698,30 +7029,211 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
+          <t>Víctor Adiel Luján</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Product Owner / backend</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>12:07</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Proveedor nuevo con RUC o DNI (decisión D-C5) y decisiones de la API ratificadas (commit)</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>HU-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Día 8</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Víctor Adiel Luján</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Product Owner / backend</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Diagramas en draw.io editable; PR #2 fusionado a main</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Base de datos</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Día 8</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Equipo Scrum</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Scrum Team</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr"/>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Presentación al docente: puntuación de las HU, objetivo del sprint y tarjetas DoR y DoD; se recibe su retroalimentación</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Product Backlog y Sprint Backlog</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Día 8</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
           <t>Fernando Istaña</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>Scrum Master</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr"/>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>Auditoría de coherencia y SWEBOK; tablero Scrum con las tareas por HU y responsables</t>
-        </is>
-      </c>
-      <c r="H20" s="7" t="inlineStr">
-        <is>
-          <t>T-239</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>La columna «Hora» la completa cada colaborador con la hora real de su actividad; desde aquí cada uno agrega una fila por actividad del día.</t>
+      <c r="F23" s="7" t="inlineStr"/>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Auditoría de coherencia y SWEBOK; corrección de 7 errores en los diagramas</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Modelado UML</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Día 8</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Fernando Istaña</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Scrum Master</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>22:08</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Tablero Scrum con las tareas por HU y guía de arranque de Henry en la web (commit en la rama scrum-tablero-sprint-1)</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>T-253</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Día 8</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Fernando Istaña</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Scrum Master</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Tareas con el modelo del docente, registro de incidencias, bitácora e historias técnicas HT-01 a HT-08 (commit)</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>T-253</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>Las horas son las de los commits del repositorio. Donde la hora está vacía, la completa el colaborador; desde aquí cada uno agrega una fila por actividad del día.</t>
         </is>
       </c>
     </row>

</xml_diff>